<commit_message>
update WR dashboard data 2026-07-01 12:44
</commit_message>
<xml_diff>
--- a/docs/reports/daily/WR_Kavach_Unified_KPI_Jun29-Jun29.xlsx
+++ b/docs/reports/daily/WR_Kavach_Unified_KPI_Jun29-Jun29.xlsx
@@ -1,18 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unified KPI" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Daily Breakdown" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EB Detail" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mode Degradation" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KM Verification" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Methodology" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Unified KPI" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Daily Breakdown" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="EB Detail" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Mode Degradation" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="KM Verification" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Methodology" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -3618,7 +3618,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L122"/>
+  <dimension ref="A1:M122"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3696,6 +3696,11 @@
           <t>Valid Trip?</t>
         </is>
       </c>
+      <c r="M5" s="14" t="inlineStr">
+        <is>
+          <t>Loco Travel</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="31" t="inlineStr">
@@ -3752,6 +3757,7 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M6" s="16" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="31" t="inlineStr">
@@ -3808,6 +3814,7 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M7" s="16" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="31" t="inlineStr">
@@ -3864,6 +3871,7 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M8" s="16" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="16" t="inlineStr">
@@ -3920,6 +3928,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M9" s="16" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="16" t="inlineStr">
@@ -3976,6 +3985,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M10" s="16" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="16" t="inlineStr">
@@ -4032,6 +4042,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M11" s="16" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="16" t="inlineStr">
@@ -4088,6 +4099,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M12" s="16" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="16" t="inlineStr">
@@ -4144,6 +4156,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M13" s="16" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="16" t="inlineStr">
@@ -4200,6 +4213,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M14" s="16" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="16" t="inlineStr">
@@ -4256,6 +4270,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M15" s="16" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="16" t="inlineStr">
@@ -4312,6 +4327,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M16" s="16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="16" t="inlineStr">
@@ -4368,6 +4384,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M17" s="16" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="16" t="inlineStr">
@@ -4424,6 +4441,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M18" s="16" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="16" t="inlineStr">
@@ -4480,6 +4498,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M19" s="16" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="31" t="inlineStr">
@@ -4536,6 +4555,7 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M20" s="16" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="16" t="inlineStr">
@@ -4592,6 +4612,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M21" s="16" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="16" t="inlineStr">
@@ -4648,6 +4669,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M22" s="16" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="31" t="inlineStr">
@@ -4704,6 +4726,7 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M23" s="16" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="31" t="inlineStr">
@@ -4760,6 +4783,7 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M24" s="16" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="16" t="inlineStr">
@@ -4816,6 +4840,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M25" s="16" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="16" t="inlineStr">
@@ -4872,6 +4897,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M26" s="16" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="16" t="inlineStr">
@@ -4928,6 +4954,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M27" s="16" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="31" t="inlineStr">
@@ -4984,6 +5011,7 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M28" s="16" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="31" t="inlineStr">
@@ -5040,6 +5068,7 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M29" s="16" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="31" t="inlineStr">
@@ -5096,6 +5125,7 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M30" s="16" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="31" t="inlineStr">
@@ -5152,6 +5182,7 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M31" s="16" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="31" t="inlineStr">
@@ -5208,6 +5239,7 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M32" s="16" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="16" t="inlineStr">
@@ -5264,6 +5296,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M33" s="16" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="16" t="inlineStr">
@@ -5320,6 +5353,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M34" s="16" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="16" t="inlineStr">
@@ -5376,6 +5410,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M35" s="16" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="16" t="inlineStr">
@@ -5432,6 +5467,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M36" s="16" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="16" t="inlineStr">
@@ -5488,6 +5524,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M37" s="16" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="16" t="inlineStr">
@@ -5544,6 +5581,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M38" s="16" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="16" t="inlineStr">
@@ -5600,6 +5638,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M39" s="16" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" s="16" t="inlineStr">
@@ -5656,6 +5695,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M40" s="16" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" s="16" t="inlineStr">
@@ -5712,6 +5752,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M41" s="16" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" s="16" t="inlineStr">
@@ -5768,6 +5809,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M42" s="16" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" s="16" t="inlineStr">
@@ -5824,6 +5866,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M43" s="16" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" s="16" t="inlineStr">
@@ -5880,6 +5923,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M44" s="16" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" s="16" t="inlineStr">
@@ -5936,6 +5980,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M45" s="16" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" s="16" t="inlineStr">
@@ -5992,6 +6037,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M46" s="16" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" s="16" t="inlineStr">
@@ -6048,6 +6094,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M47" s="16" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" s="16" t="inlineStr">
@@ -6104,6 +6151,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M48" s="16" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" s="16" t="inlineStr">
@@ -6160,6 +6208,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M49" s="16" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" s="16" t="inlineStr">
@@ -6216,6 +6265,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M50" s="16" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" s="16" t="inlineStr">
@@ -6272,6 +6322,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M51" s="16" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" s="16" t="inlineStr">
@@ -6328,6 +6379,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M52" s="16" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" s="16" t="inlineStr">
@@ -6384,6 +6436,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M53" s="16" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" s="16" t="inlineStr">
@@ -6440,6 +6493,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M54" s="16" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" s="16" t="inlineStr">
@@ -6496,6 +6550,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M55" s="16" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" s="16" t="inlineStr">
@@ -6552,6 +6607,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M56" s="16" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" s="16" t="inlineStr">
@@ -6608,6 +6664,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M57" s="16" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" s="16" t="inlineStr">
@@ -6664,6 +6721,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M58" s="16" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" s="31" t="inlineStr">
@@ -6720,6 +6778,7 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M59" s="16" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" s="16" t="inlineStr">
@@ -6776,6 +6835,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M60" s="16" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" s="16" t="inlineStr">
@@ -6832,6 +6892,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M61" s="16" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" s="16" t="inlineStr">
@@ -6888,6 +6949,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M62" s="16" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" s="16" t="inlineStr">
@@ -6944,6 +7006,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M63" s="16" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" s="16" t="inlineStr">
@@ -7000,6 +7063,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M64" s="16" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" s="16" t="inlineStr">
@@ -7056,6 +7120,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M65" s="16" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" s="16" t="inlineStr">
@@ -7112,6 +7177,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M66" s="16" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" s="16" t="inlineStr">
@@ -7168,6 +7234,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M67" s="16" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" s="16" t="inlineStr">
@@ -7224,6 +7291,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M68" s="16" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" s="16" t="inlineStr">
@@ -7280,6 +7348,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M69" s="16" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" s="31" t="inlineStr">
@@ -7336,6 +7405,7 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M70" s="16" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" s="31" t="inlineStr">
@@ -7392,6 +7462,7 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M71" s="16" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" s="31" t="inlineStr">
@@ -7448,6 +7519,7 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M72" s="16" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" s="31" t="inlineStr">
@@ -7504,6 +7576,7 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M73" s="16" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" s="16" t="inlineStr">
@@ -7560,6 +7633,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M74" s="16" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" s="31" t="inlineStr">
@@ -7616,6 +7690,7 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M75" s="16" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" s="31" t="inlineStr">
@@ -7672,6 +7747,7 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M76" s="16" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" s="31" t="inlineStr">
@@ -7728,6 +7804,7 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M77" s="16" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" s="31" t="inlineStr">
@@ -7784,6 +7861,7 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M78" s="16" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" s="31" t="inlineStr">
@@ -7840,6 +7918,7 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M79" s="16" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" s="16" t="inlineStr">
@@ -7896,6 +7975,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M80" s="16" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" s="31" t="inlineStr">
@@ -7952,6 +8032,7 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M81" s="16" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" s="16" t="inlineStr">
@@ -8008,6 +8089,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M82" s="16" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" s="16" t="inlineStr">
@@ -8064,6 +8146,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M83" s="16" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" s="16" t="inlineStr">
@@ -8120,6 +8203,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M84" s="16" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" s="16" t="inlineStr">
@@ -8176,6 +8260,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M85" s="16" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" s="16" t="inlineStr">
@@ -8232,6 +8317,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M86" s="16" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" s="16" t="inlineStr">
@@ -8288,6 +8374,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M87" s="16" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" s="31" t="inlineStr">
@@ -8344,6 +8431,7 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M88" s="16" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" s="16" t="inlineStr">
@@ -8400,6 +8488,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M89" s="16" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" s="16" t="inlineStr">
@@ -8456,6 +8545,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M90" s="16" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" s="16" t="inlineStr">
@@ -8512,6 +8602,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M91" s="16" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" s="31" t="inlineStr">
@@ -8568,6 +8659,7 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M92" s="16" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" s="31" t="inlineStr">
@@ -8624,6 +8716,7 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M93" s="16" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" s="31" t="inlineStr">
@@ -8680,6 +8773,7 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M94" s="16" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" s="16" t="inlineStr">
@@ -8736,6 +8830,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M95" s="16" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" s="16" t="inlineStr">
@@ -8792,6 +8887,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M96" s="16" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" s="16" t="inlineStr">
@@ -8848,6 +8944,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M97" s="16" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" s="16" t="inlineStr">
@@ -8904,6 +9001,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M98" s="16" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" s="16" t="inlineStr">
@@ -8960,6 +9058,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M99" s="16" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" s="16" t="inlineStr">
@@ -9016,6 +9115,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M100" s="16" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" s="16" t="inlineStr">
@@ -9072,6 +9172,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M101" s="16" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" s="16" t="inlineStr">
@@ -9128,6 +9229,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M102" s="16" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" s="16" t="inlineStr">
@@ -9184,6 +9286,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M103" s="16" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" s="16" t="inlineStr">
@@ -9240,6 +9343,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M104" s="16" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" s="16" t="inlineStr">
@@ -9296,6 +9400,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M105" s="16" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" s="16" t="inlineStr">
@@ -9352,6 +9457,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M106" s="16" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" s="16" t="inlineStr">
@@ -9408,6 +9514,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M107" s="16" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" s="16" t="inlineStr">
@@ -9464,6 +9571,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M108" s="16" t="inlineStr"/>
     </row>
     <row r="109">
       <c r="A109" s="16" t="inlineStr">
@@ -9520,6 +9628,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M109" s="16" t="inlineStr"/>
     </row>
     <row r="110">
       <c r="A110" s="16" t="inlineStr">
@@ -9576,6 +9685,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M110" s="16" t="inlineStr"/>
     </row>
     <row r="111">
       <c r="A111" s="16" t="inlineStr">
@@ -9632,6 +9742,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M111" s="16" t="inlineStr"/>
     </row>
     <row r="112">
       <c r="A112" s="31" t="inlineStr">
@@ -9688,6 +9799,7 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M112" s="16" t="inlineStr"/>
     </row>
     <row r="113">
       <c r="A113" s="16" t="inlineStr">
@@ -9744,6 +9856,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M113" s="16" t="inlineStr"/>
     </row>
     <row r="114">
       <c r="A114" s="16" t="inlineStr">
@@ -9800,6 +9913,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M114" s="16" t="inlineStr"/>
     </row>
     <row r="115">
       <c r="A115" s="31" t="inlineStr">
@@ -9856,6 +9970,7 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M115" s="16" t="inlineStr"/>
     </row>
     <row r="116">
       <c r="A116" s="31" t="inlineStr">
@@ -9912,6 +10027,7 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M116" s="16" t="inlineStr"/>
     </row>
     <row r="117">
       <c r="A117" s="31" t="inlineStr">
@@ -9968,6 +10084,7 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M117" s="16" t="inlineStr"/>
     </row>
     <row r="118">
       <c r="A118" s="16" t="inlineStr">
@@ -10024,6 +10141,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M118" s="16" t="inlineStr"/>
     </row>
     <row r="119">
       <c r="A119" s="31" t="inlineStr">
@@ -10080,6 +10198,7 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M119" s="16" t="inlineStr"/>
     </row>
     <row r="120">
       <c r="A120" s="16" t="inlineStr">
@@ -10136,6 +10255,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M120" s="16" t="inlineStr"/>
     </row>
     <row r="121">
       <c r="A121" s="16" t="inlineStr">
@@ -10192,6 +10312,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M121" s="16" t="inlineStr"/>
     </row>
     <row r="122">
       <c r="A122" s="16" t="inlineStr">
@@ -10248,6 +10369,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M122" s="16" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>

<commit_message>
update WR dashboard data 2026-07-01 13:00
</commit_message>
<xml_diff>
--- a/docs/reports/daily/WR_Kavach_Unified_KPI_Jun29-Jun29.xlsx
+++ b/docs/reports/daily/WR_Kavach_Unified_KPI_Jun29-Jun29.xlsx
@@ -3757,7 +3757,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
-      <c r="M6" s="16" t="inlineStr"/>
+      <c r="M6" s="16" t="inlineStr">
+        <is>
+          <t>BAJWA, RANOLI, LC-246, VASAD, ADAS ROAD, VADOD, LC-258, ANAND Jn, LC-264, KANJARI BORIYAVI, UTARSANDA</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="31" t="inlineStr">
@@ -3814,7 +3818,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
-      <c r="M7" s="16" t="inlineStr"/>
+      <c r="M7" s="16" t="inlineStr">
+        <is>
+          <t>BAJWA, RANOLI, LC-246, VASAD, ADAS ROAD, VADOD, LC-258, ANAND Jn, LC-264, KANJARI BORIYAVI, UTARSANDA</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="31" t="inlineStr">
@@ -3871,7 +3879,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
-      <c r="M8" s="16" t="inlineStr"/>
+      <c r="M8" s="16" t="inlineStr">
+        <is>
+          <t>BAJWA, RANOLI, LC-246, VASAD, ADAS ROAD, VADOD, LC-258, ANAND Jn, LC-264, KANJARI BORIYAVI, UTARSANDA, NADIAD</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="16" t="inlineStr">
@@ -3928,7 +3940,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M9" s="16" t="inlineStr"/>
+      <c r="M9" s="16" t="inlineStr">
+        <is>
+          <t>BAJWA, RANOLI, LC-246, VASAD, ADAS ROAD, VADOD, LC-258, ANAND Jn, LC-264, KANJARI BORIYAVI, UTARSANDA, NADIAD, LC-278, GOTHAJ, LC-286, MAHEMDABAD AND KHEDA ROAD, LC-294, KANIJ, BAREJADI NANDEJ, GERATPUR, VATVA, KANKARIYA CABIN, AHMEDABAD Jn</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="16" t="inlineStr">
@@ -3985,7 +4001,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M10" s="16" t="inlineStr"/>
+      <c r="M10" s="16" t="inlineStr">
+        <is>
+          <t>BAJWA, RANOLI, LC-246, VASAD, ADAS ROAD, VADOD, LC-258, ANAND Jn, LC-264, KANJARI BORIYAVI, UTARSANDA, NADIAD, LC-278, GOTHAJ, LC-286, MAHEMDABAD AND KHEDA ROAD, LC-294, KANIJ, BAREJADI NANDEJ, GERATPUR, VATVA, KANKARIYA CABIN, AHMEDABAD Jn</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="16" t="inlineStr">
@@ -4042,7 +4062,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M11" s="16" t="inlineStr"/>
+      <c r="M11" s="16" t="inlineStr">
+        <is>
+          <t>BAJWA, RANOLI, LC-246, VASAD, ADAS ROAD, VADOD, LC-258, ANAND Jn, LC-264, KANJARI BORIYAVI, UTARSANDA, NADIAD, LC-278, GOTHAJ, LC-286, MAHEMDABAD AND KHEDA ROAD, LC-294, KANIJ, BAREJADI NANDEJ, GERATPUR, VATVA, KANKARIYA CABIN, AHMEDABAD Jn</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="16" t="inlineStr">
@@ -4099,7 +4123,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M12" s="16" t="inlineStr"/>
+      <c r="M12" s="16" t="inlineStr">
+        <is>
+          <t>BAJWA, RANOLI, LC-246, VASAD, ADAS ROAD, VADOD, LC-258, ANAND Jn, LC-264, KANJARI BORIYAVI, UTARSANDA, NADIAD, LC-278, GOTHAJ, LC-286, MAHEMDABAD AND KHEDA ROAD, LC-294, KANIJ, BAREJADI NANDEJ, GERATPUR, VATVA, KANKARIYA CABIN, AHMEDABAD Jn</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="16" t="inlineStr">
@@ -4156,7 +4184,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M13" s="16" t="inlineStr"/>
+      <c r="M13" s="16" t="inlineStr">
+        <is>
+          <t>BAJWA, RANOLI, LC-246, VASAD, ADAS ROAD, VADOD, LC-258, ANAND Jn, LC-264, KANJARI BORIYAVI, UTARSANDA, NADIAD, LC-278, GOTHAJ, LC-286, MAHEMDABAD AND KHEDA ROAD, LC-294, KANIJ, BAREJADI NANDEJ, GERATPUR, VATVA, KANKARIYA CABIN, AHMEDABAD Jn</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="16" t="inlineStr">
@@ -4213,7 +4245,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M14" s="16" t="inlineStr"/>
+      <c r="M14" s="16" t="inlineStr">
+        <is>
+          <t>BAJWA, RANOLI, LC-246, VASAD, ADAS ROAD, VADOD, LC-258, ANAND Jn, LC-264, KANJARI BORIYAVI, UTARSANDA, NADIAD, LC-278, GOTHAJ, LC-286, MAHEMDABAD AND KHEDA ROAD, LC-294, KANIJ, BAREJADI NANDEJ, GERATPUR, VATVA, KANKARIYA CABIN, AHMEDABAD Jn</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="16" t="inlineStr">
@@ -4270,7 +4306,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M15" s="16" t="inlineStr"/>
+      <c r="M15" s="16" t="inlineStr">
+        <is>
+          <t>BAJWA, RANOLI, LC-246, VASAD, ADAS ROAD, VADOD, LC-258, ANAND Jn, LC-264, KANJARI BORIYAVI, UTARSANDA, NADIAD, LC-278, GOTHAJ, LC-286, MAHEMDABAD AND KHEDA ROAD, LC-294, KANIJ, BAREJADI NANDEJ, GERATPUR, VATVA, KANKARIYA CABIN, AHMEDABAD Jn</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="16" t="inlineStr">
@@ -4327,7 +4367,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M16" s="16" t="inlineStr"/>
+      <c r="M16" s="16" t="inlineStr">
+        <is>
+          <t>BAJWA, RANOLI, LC-246, VASAD, ADAS ROAD, VADOD, LC-258, ANAND Jn, LC-264, KANJARI BORIYAVI, UTARSANDA, NADIAD, LC-278, GOTHAJ, LC-286, MAHEMDABAD AND KHEDA ROAD, LC-294, KANIJ, BAREJADI NANDEJ, GERATPUR, VATVA, KANKARIYA CABIN, AHMEDABAD Jn</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="16" t="inlineStr">
@@ -4384,7 +4428,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M17" s="16" t="inlineStr"/>
+      <c r="M17" s="16" t="inlineStr">
+        <is>
+          <t>BAJWA, RANOLI, LC-246, VASAD, ADAS ROAD, VADOD, LC-258, ANAND Jn, LC-264, KANJARI BORIYAVI, UTARSANDA, NADIAD, LC-278, GOTHAJ, LC-286, MAHEMDABAD AND KHEDA ROAD, LC-294, KANIJ, BAREJADI NANDEJ, GERATPUR, VATVA, KANKARIYA CABIN, AHMEDABAD Jn</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="16" t="inlineStr">
@@ -4441,7 +4489,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M18" s="16" t="inlineStr"/>
+      <c r="M18" s="16" t="inlineStr">
+        <is>
+          <t>BAJWA, RANOLI, LC-246, VASAD, ADAS ROAD, VADOD, LC-258, ANAND Jn, LC-264, KANJARI BORIYAVI, UTARSANDA, NADIAD, LC-278, GOTHAJ, LC-286, MAHEMDABAD AND KHEDA ROAD, LC-294, KANIJ, BAREJADI NANDEJ, GERATPUR, VATVA, KANKARIYA CABIN, AHMEDABAD Jn</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="16" t="inlineStr">
@@ -4498,7 +4550,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M19" s="16" t="inlineStr"/>
+      <c r="M19" s="16" t="inlineStr">
+        <is>
+          <t>BAJWA, RANOLI, LC-246, VASAD, ADAS ROAD, VADOD, LC-258, ANAND Jn, LC-264, KANJARI BORIYAVI, UTARSANDA, NADIAD, LC-278, GOTHAJ, LC-286, MAHEMDABAD AND KHEDA ROAD, LC-294, KANIJ, BAREJADI NANDEJ, GERATPUR, VATVA, KANKARIYA CABIN, AHMEDABAD Jn</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="31" t="inlineStr">
@@ -4555,7 +4611,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
-      <c r="M20" s="16" t="inlineStr"/>
+      <c r="M20" s="16" t="inlineStr">
+        <is>
+          <t>BAJWA, RANOLI, LC-246, VASAD, ADAS ROAD, VADOD, LC-258, ANAND Jn, LC-264, KANJARI BORIYAVI</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="16" t="inlineStr">
@@ -4612,7 +4672,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M21" s="16" t="inlineStr"/>
+      <c r="M21" s="16" t="inlineStr">
+        <is>
+          <t>BAJWA, RANOLI, LC-246, VASAD, ADAS ROAD, VADOD, LC-258, ANAND Jn, LC-264, KANJARI BORIYAVI, UTARSANDA, NADIAD, LC-278, GOTHAJ, LC-286, MAHEMDABAD AND KHEDA ROAD, LC-294, KANIJ, BAREJADI NANDEJ, GERATPUR, VATVA, KANKARIYA CABIN, AHMEDABAD Jn</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="16" t="inlineStr">
@@ -4669,7 +4733,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M22" s="16" t="inlineStr"/>
+      <c r="M22" s="16" t="inlineStr">
+        <is>
+          <t>BAJWA, RANOLI, LC-246, VASAD, ADAS ROAD, VADOD, LC-258, ANAND Jn, LC-264, KANJARI BORIYAVI, UTARSANDA, NADIAD, LC-278, GOTHAJ, LC-286, MAHEMDABAD AND KHEDA ROAD, LC-294, KANIJ, BAREJADI NANDEJ, GERATPUR, VATVA, KANKARIYA CABIN, AHMEDABAD Jn</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="31" t="inlineStr">
@@ -4726,7 +4794,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
-      <c r="M23" s="16" t="inlineStr"/>
+      <c r="M23" s="16" t="inlineStr">
+        <is>
+          <t>ANAND Jn, LC-264, KANJARI BORIYAVI, UTARSANDA, NADIAD, LC-278, GOTHAJ, LC-286, MAHEMDABAD AND KHEDA ROAD, LC-294, KANIJ, BAREJADI NANDEJ, GERATPUR, VATVA, KANKARIYA CABIN, AHMEDABAD Jn</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="31" t="inlineStr">
@@ -4783,7 +4855,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
-      <c r="M24" s="16" t="inlineStr"/>
+      <c r="M24" s="16" t="inlineStr">
+        <is>
+          <t>ANAND Jn, LC-264, KANJARI BORIYAVI, UTARSANDA, NADIAD, LC-278, GOTHAJ, LC-286, MAHEMDABAD AND KHEDA ROAD, LC-294, KANIJ, BAREJADI NANDEJ, GERATPUR, VATVA, KANKARIYA CABIN, AHMEDABAD Jn</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="16" t="inlineStr">
@@ -4840,7 +4916,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M25" s="16" t="inlineStr"/>
+      <c r="M25" s="16" t="inlineStr">
+        <is>
+          <t>BAJWA, RANOLI, LC-246, VASAD, ADAS ROAD, VADOD, LC-258, ANAND Jn, LC-264, KANJARI BORIYAVI, UTARSANDA, NADIAD, LC-278, GOTHAJ, LC-286, MAHEMDABAD AND KHEDA ROAD, LC-294, KANIJ, BAREJADI NANDEJ, GERATPUR, VATVA, KANKARIYA CABIN, AHMEDABAD Jn</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="16" t="inlineStr">
@@ -4897,7 +4977,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M26" s="16" t="inlineStr"/>
+      <c r="M26" s="16" t="inlineStr">
+        <is>
+          <t>BAJWA, RANOLI, LC-246, VASAD, ADAS ROAD, VADOD, LC-258, ANAND Jn, LC-264, KANJARI BORIYAVI, UTARSANDA, NADIAD, LC-278, GOTHAJ, LC-286, MAHEMDABAD AND KHEDA ROAD, LC-294, KANIJ, BAREJADI NANDEJ, GERATPUR, VATVA, KANKARIYA CABIN, AHMEDABAD Jn</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="16" t="inlineStr">
@@ -4954,7 +5038,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M27" s="16" t="inlineStr"/>
+      <c r="M27" s="16" t="inlineStr">
+        <is>
+          <t>BAJWA, RANOLI, LC-246, VASAD, ADAS ROAD, VADOD, LC-258, ANAND Jn, LC-264, KANJARI BORIYAVI, UTARSANDA, NADIAD, LC-278, GOTHAJ, LC-286, MAHEMDABAD AND KHEDA ROAD, LC-294, KANIJ, BAREJADI NANDEJ, GERATPUR, VATVA, KANKARIYA CABIN, AHMEDABAD Jn</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="31" t="inlineStr">
@@ -5011,7 +5099,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
-      <c r="M28" s="16" t="inlineStr"/>
+      <c r="M28" s="16" t="inlineStr">
+        <is>
+          <t>ANAND Jn, LC-264, KANJARI BORIYAVI, UTARSANDA, NADIAD, LC-278, GOTHAJ, LC-286, MAHEMDABAD AND KHEDA ROAD, LC-294, KANIJ, BAREJADI NANDEJ, GERATPUR, VATVA, KANKARIYA CABIN, AHMEDABAD Jn</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="31" t="inlineStr">
@@ -5068,7 +5160,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
-      <c r="M29" s="16" t="inlineStr"/>
+      <c r="M29" s="16" t="inlineStr">
+        <is>
+          <t>ANAND Jn, LC-264, KANJARI BORIYAVI, UTARSANDA, NADIAD, LC-278, GOTHAJ, LC-286, MAHEMDABAD AND KHEDA ROAD, LC-294, KANIJ, BAREJADI NANDEJ, GERATPUR, VATVA, KANKARIYA CABIN, AHMEDABAD Jn</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="31" t="inlineStr">
@@ -5125,7 +5221,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
-      <c r="M30" s="16" t="inlineStr"/>
+      <c r="M30" s="16" t="inlineStr">
+        <is>
+          <t>ANAND Jn, LC-264, KANJARI BORIYAVI, UTARSANDA, NADIAD, LC-278, GOTHAJ, LC-286, MAHEMDABAD AND KHEDA ROAD, LC-294, KANIJ, BAREJADI NANDEJ, GERATPUR, VATVA, KANKARIYA CABIN, AHMEDABAD Jn</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="31" t="inlineStr">
@@ -5182,7 +5282,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
-      <c r="M31" s="16" t="inlineStr"/>
+      <c r="M31" s="16" t="inlineStr">
+        <is>
+          <t>BAJWA, RANOLI, LC-246, VASAD, ADAS ROAD, VADOD, LC-258, ANAND Jn, LC-264, KANJARI BORIYAVI, UTARSANDA</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="31" t="inlineStr">
@@ -5239,7 +5343,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
-      <c r="M32" s="16" t="inlineStr"/>
+      <c r="M32" s="16" t="inlineStr">
+        <is>
+          <t>ANAND Jn, LC-264, KANJARI BORIYAVI, UTARSANDA, NADIAD, LC-278, GOTHAJ, LC-286, MAHEMDABAD AND KHEDA ROAD, LC-294, KANIJ, BAREJADI NANDEJ, GERATPUR, VATVA, KANKARIYA CABIN, AHMEDABAD Jn</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="16" t="inlineStr">
@@ -5296,7 +5404,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M33" s="16" t="inlineStr"/>
+      <c r="M33" s="16" t="inlineStr">
+        <is>
+          <t>BAJWA, RANOLI, LC-246, VASAD, ADAS ROAD, VADOD, LC-258, ANAND Jn, LC-264, KANJARI BORIYAVI, UTARSANDA, NADIAD, LC-278, GOTHAJ, LC-286, MAHEMDABAD AND KHEDA ROAD, LC-294, KANIJ, BAREJADI NANDEJ, GERATPUR, VATVA, KANKARIYA CABIN, AHMEDABAD Jn</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="16" t="inlineStr">
@@ -5353,7 +5465,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M34" s="16" t="inlineStr"/>
+      <c r="M34" s="16" t="inlineStr">
+        <is>
+          <t>BAJWA, RANOLI, LC-246, VASAD, ADAS ROAD, VADOD, LC-258, ANAND Jn, LC-264, KANJARI BORIYAVI, UTARSANDA, NADIAD, LC-278, GOTHAJ, LC-286, MAHEMDABAD AND KHEDA ROAD, LC-294, KANIJ, BAREJADI NANDEJ, GERATPUR, VATVA, KANKARIYA CABIN, AHMEDABAD Jn</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="16" t="inlineStr">
@@ -5410,7 +5526,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M35" s="16" t="inlineStr"/>
+      <c r="M35" s="16" t="inlineStr">
+        <is>
+          <t>BAJWA, RANOLI, LC-246, VASAD, ADAS ROAD, VADOD, LC-258, ANAND Jn, LC-264, KANJARI BORIYAVI, UTARSANDA, NADIAD, LC-278, GOTHAJ, LC-286, MAHEMDABAD AND KHEDA ROAD, LC-294, KANIJ, BAREJADI NANDEJ, GERATPUR, VATVA, KANKARIYA CABIN, AHMEDABAD Jn</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="16" t="inlineStr">
@@ -5467,7 +5587,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M36" s="16" t="inlineStr"/>
+      <c r="M36" s="16" t="inlineStr">
+        <is>
+          <t>BAJWA, RANOLI, LC-246, VASAD, ADAS ROAD, VADOD, LC-258, ANAND Jn, LC-264, KANJARI BORIYAVI, UTARSANDA, NADIAD, LC-278, GOTHAJ, LC-286, MAHEMDABAD AND KHEDA ROAD, LC-294, KANIJ, BAREJADI NANDEJ, GERATPUR, VATVA, KANKARIYA CABIN, AHMEDABAD Jn</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="16" t="inlineStr">
@@ -5524,7 +5648,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M37" s="16" t="inlineStr"/>
+      <c r="M37" s="16" t="inlineStr">
+        <is>
+          <t>BAJWA, RANOLI, LC-246, VASAD, ADAS ROAD, VADOD, LC-258, ANAND Jn, LC-264, KANJARI BORIYAVI, UTARSANDA, NADIAD, LC-278, GOTHAJ, LC-286, MAHEMDABAD AND KHEDA ROAD, LC-294, KANIJ, BAREJADI NANDEJ, GERATPUR, VATVA, KANKARIYA CABIN, AHMEDABAD Jn</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="16" t="inlineStr">
@@ -5581,7 +5709,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M38" s="16" t="inlineStr"/>
+      <c r="M38" s="16" t="inlineStr">
+        <is>
+          <t>BAJWA, RANOLI, LC-246, VASAD, ADAS ROAD, VADOD, LC-258, ANAND Jn, LC-264, KANJARI BORIYAVI, UTARSANDA, NADIAD, LC-278, GOTHAJ, LC-286, MAHEMDABAD AND KHEDA ROAD, LC-294, KANIJ, BAREJADI NANDEJ, GERATPUR, VATVA, KANKARIYA CABIN, AHMEDABAD Jn</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="16" t="inlineStr">
@@ -5638,7 +5770,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M39" s="16" t="inlineStr"/>
+      <c r="M39" s="16" t="inlineStr">
+        <is>
+          <t>BAJWA, RANOLI, LC-246, VASAD, ADAS ROAD, VADOD, LC-258, ANAND Jn, LC-264, KANJARI BORIYAVI, UTARSANDA, NADIAD, LC-278, GOTHAJ, LC-286, MAHEMDABAD AND KHEDA ROAD, LC-294, KANIJ, BAREJADI NANDEJ, GERATPUR, VATVA, KANKARIYA CABIN, AHMEDABAD Jn</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="16" t="inlineStr">
@@ -5695,7 +5831,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M40" s="16" t="inlineStr"/>
+      <c r="M40" s="16" t="inlineStr">
+        <is>
+          <t>BAJWA, RANOLI, LC-246, VASAD, ADAS ROAD, VADOD, LC-258, ANAND Jn, LC-264, KANJARI BORIYAVI, UTARSANDA, NADIAD, LC-278, GOTHAJ, LC-286, MAHEMDABAD AND KHEDA ROAD, LC-294, KANIJ, BAREJADI NANDEJ, GERATPUR, VATVA, KANKARIYA CABIN, AHMEDABAD Jn</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="16" t="inlineStr">
@@ -5752,7 +5892,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M41" s="16" t="inlineStr"/>
+      <c r="M41" s="16" t="inlineStr">
+        <is>
+          <t>BAJWA, RANOLI, LC-246, VASAD, ADAS ROAD, VADOD, LC-258, ANAND Jn, LC-264, KANJARI BORIYAVI, UTARSANDA, NADIAD, LC-278, GOTHAJ, LC-286, MAHEMDABAD AND KHEDA ROAD, LC-294, KANIJ, BAREJADI NANDEJ, GERATPUR, VATVA, KANKARIYA CABIN, AHMEDABAD Jn</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="16" t="inlineStr">
@@ -5809,7 +5953,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M42" s="16" t="inlineStr"/>
+      <c r="M42" s="16" t="inlineStr">
+        <is>
+          <t>BAJWA, RANOLI, LC-246, VASAD, ADAS ROAD, VADOD, LC-258, ANAND Jn, LC-264, KANJARI BORIYAVI, UTARSANDA, NADIAD, LC-278, GOTHAJ, LC-286, MAHEMDABAD AND KHEDA ROAD, LC-294, KANIJ, BAREJADI NANDEJ, GERATPUR, VATVA, KANKARIYA CABIN, AHMEDABAD Jn</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="16" t="inlineStr">
@@ -5866,7 +6014,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M43" s="16" t="inlineStr"/>
+      <c r="M43" s="16" t="inlineStr">
+        <is>
+          <t>BAJWA, RANOLI, LC-246, VASAD, ADAS ROAD, VADOD, LC-258, ANAND Jn, LC-264, KANJARI BORIYAVI, UTARSANDA, NADIAD, LC-278, GOTHAJ, LC-286, MAHEMDABAD AND KHEDA ROAD, LC-294, KANIJ, BAREJADI NANDEJ, GERATPUR, VATVA, KANKARIYA CABIN, AHMEDABAD Jn</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="16" t="inlineStr">
@@ -5923,7 +6075,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M44" s="16" t="inlineStr"/>
+      <c r="M44" s="16" t="inlineStr">
+        <is>
+          <t>BAJWA, RANOLI, LC-246, VASAD, ADAS ROAD, VADOD, LC-258, ANAND Jn, LC-264, KANJARI BORIYAVI, UTARSANDA, NADIAD, LC-278, GOTHAJ, LC-286, MAHEMDABAD AND KHEDA ROAD, LC-294, KANIJ, BAREJADI NANDEJ, GERATPUR, VATVA, KANKARIYA CABIN, AHMEDABAD Jn</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="16" t="inlineStr">
@@ -5980,7 +6136,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M45" s="16" t="inlineStr"/>
+      <c r="M45" s="16" t="inlineStr">
+        <is>
+          <t>BAJWA, RANOLI, LC-246, VASAD, ADAS ROAD, VADOD, LC-258, ANAND Jn, LC-264, KANJARI BORIYAVI, UTARSANDA, NADIAD, LC-278, GOTHAJ, LC-286, MAHEMDABAD AND KHEDA ROAD, LC-294, KANIJ, BAREJADI NANDEJ, GERATPUR, VATVA, KANKARIYA CABIN, AHMEDABAD Jn</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="16" t="inlineStr">
@@ -6037,7 +6197,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M46" s="16" t="inlineStr"/>
+      <c r="M46" s="16" t="inlineStr">
+        <is>
+          <t>BAJWA, RANOLI, LC-246, VASAD, ADAS ROAD, VADOD, LC-258, ANAND Jn, LC-264, KANJARI BORIYAVI, UTARSANDA, NADIAD, LC-278, GOTHAJ, LC-286, MAHEMDABAD AND KHEDA ROAD, LC-294, KANIJ, BAREJADI NANDEJ, GERATPUR, VATVA, KANKARIYA CABIN, AHMEDABAD Jn</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="16" t="inlineStr">
@@ -6094,7 +6258,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M47" s="16" t="inlineStr"/>
+      <c r="M47" s="16" t="inlineStr">
+        <is>
+          <t>BAJWA, RANOLI, LC-246, VASAD, ADAS ROAD, VADOD, LC-258, ANAND Jn, LC-264, KANJARI BORIYAVI, UTARSANDA, NADIAD, LC-278, GOTHAJ, LC-286, MAHEMDABAD AND KHEDA ROAD, LC-294, KANIJ, BAREJADI NANDEJ, GERATPUR, VATVA, KANKARIYA CABIN, AHMEDABAD Jn</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="16" t="inlineStr">
@@ -6151,7 +6319,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M48" s="16" t="inlineStr"/>
+      <c r="M48" s="16" t="inlineStr">
+        <is>
+          <t>BAJWA, RANOLI, LC-246, VASAD, ADAS ROAD, VADOD, LC-258, ANAND Jn, LC-264, KANJARI BORIYAVI, UTARSANDA, NADIAD, LC-278, GOTHAJ, LC-286, MAHEMDABAD AND KHEDA ROAD, LC-294, KANIJ, BAREJADI NANDEJ, GERATPUR, VATVA, KANKARIYA CABIN, AHMEDABAD Jn</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="16" t="inlineStr">
@@ -6208,7 +6380,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M49" s="16" t="inlineStr"/>
+      <c r="M49" s="16" t="inlineStr">
+        <is>
+          <t>BAJWA, RANOLI, LC-246, VASAD, ADAS ROAD, VADOD, LC-258, ANAND Jn, LC-264, KANJARI BORIYAVI, UTARSANDA, NADIAD, LC-278, GOTHAJ, LC-286, MAHEMDABAD AND KHEDA ROAD, LC-294, KANIJ, BAREJADI NANDEJ, GERATPUR, VATVA, KANKARIYA CABIN, AHMEDABAD Jn</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="16" t="inlineStr">
@@ -6265,7 +6441,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M50" s="16" t="inlineStr"/>
+      <c r="M50" s="16" t="inlineStr">
+        <is>
+          <t>BAJWA, RANOLI, LC-246, VASAD, ADAS ROAD, VADOD, LC-258, ANAND Jn, LC-264, KANJARI BORIYAVI, UTARSANDA, NADIAD, LC-278, GOTHAJ, LC-286, MAHEMDABAD AND KHEDA ROAD, LC-294, KANIJ, BAREJADI NANDEJ, GERATPUR, VATVA, KANKARIYA CABIN, AHMEDABAD Jn</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="16" t="inlineStr">
@@ -6322,7 +6502,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M51" s="16" t="inlineStr"/>
+      <c r="M51" s="16" t="inlineStr">
+        <is>
+          <t>BAJWA, RANOLI, LC-246, VASAD, ADAS ROAD, VADOD, LC-258, ANAND Jn, LC-264, KANJARI BORIYAVI, UTARSANDA, NADIAD, LC-278, GOTHAJ, LC-286, MAHEMDABAD AND KHEDA ROAD, LC-294, KANIJ, BAREJADI NANDEJ, GERATPUR, VATVA, KANKARIYA CABIN, AHMEDABAD Jn</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="16" t="inlineStr">
@@ -6379,7 +6563,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M52" s="16" t="inlineStr"/>
+      <c r="M52" s="16" t="inlineStr">
+        <is>
+          <t>BAJWA, RANOLI, LC-246, VASAD, ADAS ROAD, VADOD, LC-258, ANAND Jn, LC-264, KANJARI BORIYAVI, UTARSANDA, NADIAD, LC-278, GOTHAJ, LC-286, MAHEMDABAD AND KHEDA ROAD, LC-294, KANIJ, BAREJADI NANDEJ, GERATPUR, VATVA, KANKARIYA CABIN, AHMEDABAD Jn</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="16" t="inlineStr">
@@ -6436,7 +6624,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M53" s="16" t="inlineStr"/>
+      <c r="M53" s="16" t="inlineStr">
+        <is>
+          <t>BAJWA, RANOLI, LC-246, VASAD, ADAS ROAD, VADOD, LC-258, ANAND Jn, LC-264, KANJARI BORIYAVI, UTARSANDA, NADIAD, LC-278, GOTHAJ, LC-286, MAHEMDABAD AND KHEDA ROAD, LC-294, KANIJ, BAREJADI NANDEJ, GERATPUR, VATVA, KANKARIYA CABIN, AHMEDABAD Jn</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="16" t="inlineStr">
@@ -6493,7 +6685,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M54" s="16" t="inlineStr"/>
+      <c r="M54" s="16" t="inlineStr">
+        <is>
+          <t>BAJWA, RANOLI, LC-246, VASAD, ADAS ROAD, VADOD, LC-258, ANAND Jn, LC-264, KANJARI BORIYAVI, UTARSANDA, NADIAD, LC-278, GOTHAJ, LC-286, MAHEMDABAD AND KHEDA ROAD, LC-294, KANIJ, BAREJADI NANDEJ, GERATPUR, VATVA, KANKARIYA CABIN, AHMEDABAD Jn</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="16" t="inlineStr">
@@ -6550,7 +6746,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M55" s="16" t="inlineStr"/>
+      <c r="M55" s="16" t="inlineStr">
+        <is>
+          <t>BAJWA, RANOLI, LC-246, VASAD, ADAS ROAD, VADOD, LC-258, ANAND Jn, LC-264, KANJARI BORIYAVI, UTARSANDA, NADIAD, LC-278, GOTHAJ, LC-286, MAHEMDABAD AND KHEDA ROAD, LC-294, KANIJ, BAREJADI NANDEJ, GERATPUR, VATVA, KANKARIYA CABIN, AHMEDABAD Jn</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="16" t="inlineStr">
@@ -6607,7 +6807,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M56" s="16" t="inlineStr"/>
+      <c r="M56" s="16" t="inlineStr">
+        <is>
+          <t>BAJWA, RANOLI, LC-246, VASAD, ADAS ROAD, VADOD, LC-258, ANAND Jn, LC-264, KANJARI BORIYAVI, UTARSANDA, NADIAD, LC-278, GOTHAJ, LC-286, MAHEMDABAD AND KHEDA ROAD, LC-294, KANIJ, BAREJADI NANDEJ, GERATPUR, VATVA, KANKARIYA CABIN, AHMEDABAD Jn</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="16" t="inlineStr">
@@ -6664,7 +6868,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M57" s="16" t="inlineStr"/>
+      <c r="M57" s="16" t="inlineStr">
+        <is>
+          <t>BAJWA, RANOLI, LC-246, VASAD, ADAS ROAD, VADOD, LC-258, ANAND Jn, LC-264, KANJARI BORIYAVI, UTARSANDA, NADIAD, LC-278, GOTHAJ, LC-286, MAHEMDABAD AND KHEDA ROAD, LC-294, KANIJ, BAREJADI NANDEJ, GERATPUR, VATVA, KANKARIYA CABIN, AHMEDABAD Jn</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="16" t="inlineStr">
@@ -6721,7 +6929,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M58" s="16" t="inlineStr"/>
+      <c r="M58" s="16" t="inlineStr">
+        <is>
+          <t>BAJWA, RANOLI, LC-246, VASAD, ADAS ROAD, VADOD, LC-258, ANAND Jn, LC-264, KANJARI BORIYAVI, UTARSANDA, NADIAD, LC-278, GOTHAJ, LC-286, MAHEMDABAD AND KHEDA ROAD, LC-294, KANIJ, BAREJADI NANDEJ, GERATPUR, VATVA, KANKARIYA CABIN, AHMEDABAD Jn</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="31" t="inlineStr">
@@ -6778,7 +6990,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
-      <c r="M59" s="16" t="inlineStr"/>
+      <c r="M59" s="16" t="inlineStr">
+        <is>
+          <t>BAJWA, RANOLI, LC-246, VASAD, ADAS ROAD, VADOD, LC-258, ANAND Jn, LC-264, KANJARI BORIYAVI</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="16" t="inlineStr">
@@ -6835,7 +7051,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M60" s="16" t="inlineStr"/>
+      <c r="M60" s="16" t="inlineStr">
+        <is>
+          <t>BAJWA, RANOLI, LC-246, VASAD, ADAS ROAD, VADOD, LC-258, ANAND Jn, LC-264, KANJARI BORIYAVI, UTARSANDA, NADIAD, LC-278, GOTHAJ, LC-286, MAHEMDABAD AND KHEDA ROAD, LC-294, KANIJ, BAREJADI NANDEJ, GERATPUR, VATVA, KANKARIYA CABIN, AHMEDABAD Jn</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="16" t="inlineStr">
@@ -6892,7 +7112,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M61" s="16" t="inlineStr"/>
+      <c r="M61" s="16" t="inlineStr">
+        <is>
+          <t>BAJWA, RANOLI, LC-246, VASAD, ADAS ROAD, VADOD, LC-258, ANAND Jn, LC-264, KANJARI BORIYAVI, UTARSANDA, NADIAD, LC-278, GOTHAJ, LC-286, MAHEMDABAD AND KHEDA ROAD, LC-294, KANIJ, BAREJADI NANDEJ, GERATPUR, VATVA, KANKARIYA CABIN, AHMEDABAD Jn</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="16" t="inlineStr">
@@ -6949,7 +7173,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M62" s="16" t="inlineStr"/>
+      <c r="M62" s="16" t="inlineStr">
+        <is>
+          <t>BAJWA, RANOLI, LC-246, VASAD, ADAS ROAD, VADOD, LC-258, ANAND Jn, LC-264, KANJARI BORIYAVI, UTARSANDA, NADIAD, LC-278, GOTHAJ, LC-286, MAHEMDABAD AND KHEDA ROAD, LC-294, KANIJ, BAREJADI NANDEJ, GERATPUR, VATVA, KANKARIYA CABIN, AHMEDABAD Jn</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="16" t="inlineStr">
@@ -7006,7 +7234,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M63" s="16" t="inlineStr"/>
+      <c r="M63" s="16" t="inlineStr">
+        <is>
+          <t>BAJWA, RANOLI, LC-246, VASAD, ADAS ROAD, VADOD, LC-258, ANAND Jn, LC-264, KANJARI BORIYAVI, UTARSANDA, NADIAD, LC-278, GOTHAJ, LC-286, MAHEMDABAD AND KHEDA ROAD, LC-294, KANIJ, BAREJADI NANDEJ, GERATPUR, VATVA, KANKARIYA CABIN, AHMEDABAD Jn</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="16" t="inlineStr">
@@ -7063,7 +7295,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M64" s="16" t="inlineStr"/>
+      <c r="M64" s="16" t="inlineStr">
+        <is>
+          <t>BAJWA, RANOLI, LC-246, VASAD, ADAS ROAD, VADOD, LC-258, ANAND Jn, LC-264, KANJARI BORIYAVI, UTARSANDA, NADIAD, LC-278, GOTHAJ, LC-286, MAHEMDABAD AND KHEDA ROAD, LC-294, KANIJ, BAREJADI NANDEJ, GERATPUR, VATVA, KANKARIYA CABIN, AHMEDABAD Jn</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="16" t="inlineStr">
@@ -7120,7 +7356,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M65" s="16" t="inlineStr"/>
+      <c r="M65" s="16" t="inlineStr">
+        <is>
+          <t>BAJWA, RANOLI, LC-246, VASAD, ADAS ROAD, VADOD, LC-258, ANAND Jn, LC-264, KANJARI BORIYAVI, UTARSANDA, NADIAD, LC-278, GOTHAJ, LC-286, MAHEMDABAD AND KHEDA ROAD, LC-294, KANIJ, BAREJADI NANDEJ, GERATPUR, VATVA, KANKARIYA CABIN, AHMEDABAD Jn</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="16" t="inlineStr">
@@ -7177,7 +7417,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M66" s="16" t="inlineStr"/>
+      <c r="M66" s="16" t="inlineStr">
+        <is>
+          <t>BAJWA, RANOLI, LC-246, VASAD, ADAS ROAD, VADOD, LC-258, ANAND Jn, LC-264, KANJARI BORIYAVI, UTARSANDA, NADIAD, LC-278, GOTHAJ, LC-286, MAHEMDABAD AND KHEDA ROAD, LC-294, KANIJ, BAREJADI NANDEJ, GERATPUR, VATVA, KANKARIYA CABIN, AHMEDABAD Jn</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="16" t="inlineStr">
@@ -7234,7 +7478,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M67" s="16" t="inlineStr"/>
+      <c r="M67" s="16" t="inlineStr">
+        <is>
+          <t>BAJWA, RANOLI, LC-246, VASAD, ADAS ROAD, VADOD, LC-258, ANAND Jn, LC-264, KANJARI BORIYAVI, UTARSANDA, NADIAD, LC-278, GOTHAJ, LC-286, MAHEMDABAD AND KHEDA ROAD, LC-294, KANIJ, BAREJADI NANDEJ, GERATPUR, VATVA, KANKARIYA CABIN, AHMEDABAD Jn</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="16" t="inlineStr">
@@ -7291,7 +7539,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M68" s="16" t="inlineStr"/>
+      <c r="M68" s="16" t="inlineStr">
+        <is>
+          <t>BAJWA, RANOLI, LC-246, VASAD, ADAS ROAD, VADOD, LC-258, ANAND Jn, LC-264, KANJARI BORIYAVI, UTARSANDA, NADIAD, LC-278, GOTHAJ, LC-286, MAHEMDABAD AND KHEDA ROAD, LC-294, KANIJ, BAREJADI NANDEJ, GERATPUR, VATVA, KANKARIYA CABIN, AHMEDABAD Jn</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="16" t="inlineStr">
@@ -7348,7 +7600,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M69" s="16" t="inlineStr"/>
+      <c r="M69" s="16" t="inlineStr">
+        <is>
+          <t>BAJWA, RANOLI, LC-246, VASAD, ADAS ROAD, VADOD, LC-258, ANAND Jn, LC-264, KANJARI BORIYAVI, UTARSANDA, NADIAD, LC-278, GOTHAJ, LC-286, MAHEMDABAD AND KHEDA ROAD, LC-294, KANIJ, BAREJADI NANDEJ, GERATPUR, VATVA, KANKARIYA CABIN, AHMEDABAD Jn</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="31" t="inlineStr">
@@ -7405,7 +7661,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
-      <c r="M70" s="16" t="inlineStr"/>
+      <c r="M70" s="16" t="inlineStr">
+        <is>
+          <t>NADIAD</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="31" t="inlineStr">
@@ -7462,7 +7722,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
-      <c r="M71" s="16" t="inlineStr"/>
+      <c r="M71" s="16" t="inlineStr">
+        <is>
+          <t>NADIAD</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="31" t="inlineStr">
@@ -7519,7 +7783,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
-      <c r="M72" s="16" t="inlineStr"/>
+      <c r="M72" s="16" t="inlineStr">
+        <is>
+          <t>BAJWA, RANOLI, LC-246, VASAD, ADAS ROAD, VADOD, LC-258, ANAND Jn, LC-264</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="31" t="inlineStr">
@@ -7576,7 +7844,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
-      <c r="M73" s="16" t="inlineStr"/>
+      <c r="M73" s="16" t="inlineStr">
+        <is>
+          <t>NADIAD</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="16" t="inlineStr">
@@ -7633,7 +7905,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M74" s="16" t="inlineStr"/>
+      <c r="M74" s="16" t="inlineStr">
+        <is>
+          <t>BAJWA, RANOLI, LC-246, VASAD, ADAS ROAD, VADOD, LC-258, ANAND Jn, LC-264, KANJARI BORIYAVI, UTARSANDA, NADIAD, LC-278, GOTHAJ, LC-286, MAHEMDABAD AND KHEDA ROAD, LC-294, KANIJ, BAREJADI NANDEJ, GERATPUR, VATVA, KANKARIYA CABIN, AHMEDABAD Jn</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="31" t="inlineStr">
@@ -7690,7 +7966,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
-      <c r="M75" s="16" t="inlineStr"/>
+      <c r="M75" s="16" t="inlineStr">
+        <is>
+          <t>NADIAD</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="31" t="inlineStr">
@@ -7747,7 +8027,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
-      <c r="M76" s="16" t="inlineStr"/>
+      <c r="M76" s="16" t="inlineStr">
+        <is>
+          <t>UTARSANDA, NADIAD</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="31" t="inlineStr">
@@ -7804,7 +8088,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
-      <c r="M77" s="16" t="inlineStr"/>
+      <c r="M77" s="16" t="inlineStr">
+        <is>
+          <t>BAJWA, RANOLI, LC-246, VASAD, ADAS ROAD, VADOD, LC-258, ANAND Jn, LC-264, KANJARI BORIYAVI</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="31" t="inlineStr">
@@ -7861,7 +8149,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
-      <c r="M78" s="16" t="inlineStr"/>
+      <c r="M78" s="16" t="inlineStr">
+        <is>
+          <t>UTARSANDA, NADIAD</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="31" t="inlineStr">
@@ -7918,7 +8210,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
-      <c r="M79" s="16" t="inlineStr"/>
+      <c r="M79" s="16" t="inlineStr">
+        <is>
+          <t>BAJWA, RANOLI, LC-246, VASAD, ADAS ROAD, VADOD, LC-258, ANAND Jn, LC-264</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="16" t="inlineStr">
@@ -7975,7 +8271,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M80" s="16" t="inlineStr"/>
+      <c r="M80" s="16" t="inlineStr">
+        <is>
+          <t>BAJWA, RANOLI, LC-246, VASAD, ADAS ROAD, VADOD, LC-258, ANAND Jn, LC-264, KANJARI BORIYAVI, UTARSANDA, NADIAD, LC-278, GOTHAJ, LC-286, MAHEMDABAD AND KHEDA ROAD, LC-294, KANIJ, BAREJADI NANDEJ, GERATPUR, VATVA, KANKARIYA CABIN, AHMEDABAD Jn</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="31" t="inlineStr">
@@ -8032,7 +8332,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
-      <c r="M81" s="16" t="inlineStr"/>
+      <c r="M81" s="16" t="inlineStr">
+        <is>
+          <t>UTARSANDA, NADIAD</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="16" t="inlineStr">
@@ -8089,7 +8393,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M82" s="16" t="inlineStr"/>
+      <c r="M82" s="16" t="inlineStr">
+        <is>
+          <t>BAJWA, RANOLI, LC-246, VASAD, ADAS ROAD, VADOD, LC-258, ANAND Jn, LC-264, KANJARI BORIYAVI, UTARSANDA, NADIAD, LC-278, GOTHAJ, LC-286, MAHEMDABAD AND KHEDA ROAD, LC-294, KANIJ, BAREJADI NANDEJ, GERATPUR, VATVA, KANKARIYA CABIN, AHMEDABAD Jn</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="16" t="inlineStr">
@@ -8146,7 +8454,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M83" s="16" t="inlineStr"/>
+      <c r="M83" s="16" t="inlineStr">
+        <is>
+          <t>BAJWA, RANOLI, LC-246, VASAD, ADAS ROAD, VADOD, LC-258, ANAND Jn, LC-264, KANJARI BORIYAVI, UTARSANDA, NADIAD, LC-278, GOTHAJ, LC-286, MAHEMDABAD AND KHEDA ROAD, LC-294, KANIJ, BAREJADI NANDEJ, GERATPUR, VATVA, KANKARIYA CABIN, AHMEDABAD Jn</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="16" t="inlineStr">
@@ -8203,7 +8515,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M84" s="16" t="inlineStr"/>
+      <c r="M84" s="16" t="inlineStr">
+        <is>
+          <t>BAJWA, RANOLI, LC-246, VASAD, ADAS ROAD, VADOD, LC-258, ANAND Jn, LC-264, KANJARI BORIYAVI, UTARSANDA, NADIAD, LC-278, GOTHAJ, LC-286, MAHEMDABAD AND KHEDA ROAD, LC-294, KANIJ, BAREJADI NANDEJ, GERATPUR, VATVA, KANKARIYA CABIN, AHMEDABAD Jn</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="16" t="inlineStr">
@@ -8260,7 +8576,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M85" s="16" t="inlineStr"/>
+      <c r="M85" s="16" t="inlineStr">
+        <is>
+          <t>BAJWA, RANOLI, LC-246, VASAD, ADAS ROAD, VADOD, LC-258, ANAND Jn, LC-264, KANJARI BORIYAVI, UTARSANDA, NADIAD, LC-278, GOTHAJ, LC-286, MAHEMDABAD AND KHEDA ROAD, LC-294, KANIJ, BAREJADI NANDEJ, GERATPUR, VATVA, KANKARIYA CABIN, AHMEDABAD Jn</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="16" t="inlineStr">
@@ -8317,7 +8637,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M86" s="16" t="inlineStr"/>
+      <c r="M86" s="16" t="inlineStr">
+        <is>
+          <t>BAJWA, RANOLI, LC-246, VASAD, ADAS ROAD, VADOD, LC-258, ANAND Jn, LC-264, KANJARI BORIYAVI, UTARSANDA, NADIAD, LC-278, GOTHAJ, LC-286, MAHEMDABAD AND KHEDA ROAD, LC-294, KANIJ, BAREJADI NANDEJ, GERATPUR, VATVA, KANKARIYA CABIN, AHMEDABAD Jn</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="16" t="inlineStr">
@@ -8374,7 +8698,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M87" s="16" t="inlineStr"/>
+      <c r="M87" s="16" t="inlineStr">
+        <is>
+          <t>BAJWA, RANOLI, LC-246, VASAD, ADAS ROAD, VADOD, LC-258, ANAND Jn, LC-264, KANJARI BORIYAVI, UTARSANDA, NADIAD, LC-278, GOTHAJ, LC-286, MAHEMDABAD AND KHEDA ROAD, LC-294, KANIJ, BAREJADI NANDEJ, GERATPUR, VATVA, KANKARIYA CABIN, AHMEDABAD Jn</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="31" t="inlineStr">
@@ -8431,7 +8759,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
-      <c r="M88" s="16" t="inlineStr"/>
+      <c r="M88" s="16" t="inlineStr">
+        <is>
+          <t>BAJWA, RANOLI, LC-246, VASAD, ADAS ROAD, VADOD, LC-258, ANAND Jn, LC-264, KANJARI BORIYAVI</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="16" t="inlineStr">
@@ -8488,7 +8820,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M89" s="16" t="inlineStr"/>
+      <c r="M89" s="16" t="inlineStr">
+        <is>
+          <t>BAJWA, RANOLI, LC-246, VASAD, ADAS ROAD, VADOD, LC-258, ANAND Jn, LC-264, KANJARI BORIYAVI, UTARSANDA, NADIAD, LC-278, GOTHAJ, LC-286, MAHEMDABAD AND KHEDA ROAD, LC-294, KANIJ, BAREJADI NANDEJ, GERATPUR, VATVA, KANKARIYA CABIN, AHMEDABAD Jn</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="16" t="inlineStr">
@@ -8545,7 +8881,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M90" s="16" t="inlineStr"/>
+      <c r="M90" s="16" t="inlineStr">
+        <is>
+          <t>BAJWA, RANOLI, LC-246, VASAD, ADAS ROAD, VADOD, LC-258, ANAND Jn, LC-264, KANJARI BORIYAVI, UTARSANDA, NADIAD, LC-278, GOTHAJ, LC-286, MAHEMDABAD AND KHEDA ROAD, LC-294, KANIJ, BAREJADI NANDEJ, GERATPUR, VATVA, KANKARIYA CABIN, AHMEDABAD Jn</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="16" t="inlineStr">
@@ -8602,7 +8942,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M91" s="16" t="inlineStr"/>
+      <c r="M91" s="16" t="inlineStr">
+        <is>
+          <t>BAJWA, RANOLI, LC-246, VASAD, ADAS ROAD, VADOD, LC-258, ANAND Jn, LC-264, KANJARI BORIYAVI, UTARSANDA, NADIAD, LC-278, GOTHAJ, LC-286, MAHEMDABAD AND KHEDA ROAD, LC-294, KANIJ, BAREJADI NANDEJ, GERATPUR, VATVA, KANKARIYA CABIN, AHMEDABAD Jn</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="31" t="inlineStr">
@@ -8659,7 +9003,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
-      <c r="M92" s="16" t="inlineStr"/>
+      <c r="M92" s="16" t="inlineStr">
+        <is>
+          <t>BAJWA, RANOLI, LC-246, VASAD, ADAS ROAD, VADOD, LC-258, ANAND Jn, LC-264, KANJARI BORIYAVI, UTARSANDA</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="31" t="inlineStr">
@@ -8716,7 +9064,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
-      <c r="M93" s="16" t="inlineStr"/>
+      <c r="M93" s="16" t="inlineStr">
+        <is>
+          <t>BAJWA, RANOLI, LC-246, VASAD, ADAS ROAD, VADOD, LC-258, ANAND Jn, LC-264, KANJARI BORIYAVI</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="31" t="inlineStr">
@@ -8773,7 +9125,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
-      <c r="M94" s="16" t="inlineStr"/>
+      <c r="M94" s="16" t="inlineStr">
+        <is>
+          <t>BAJWA, RANOLI, LC-246, VASAD, ADAS ROAD, VADOD, LC-258, ANAND Jn, LC-264, KANJARI BORIYAVI</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="16" t="inlineStr">
@@ -8830,7 +9186,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M95" s="16" t="inlineStr"/>
+      <c r="M95" s="16" t="inlineStr">
+        <is>
+          <t>BAJWA, RANOLI, LC-246, VASAD, ADAS ROAD, VADOD, LC-258, ANAND Jn, LC-264, KANJARI BORIYAVI, UTARSANDA, NADIAD, LC-278, GOTHAJ, LC-286, MAHEMDABAD AND KHEDA ROAD, LC-294, KANIJ, BAREJADI NANDEJ, GERATPUR, VATVA, KANKARIYA CABIN, AHMEDABAD Jn</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="16" t="inlineStr">
@@ -8887,7 +9247,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M96" s="16" t="inlineStr"/>
+      <c r="M96" s="16" t="inlineStr">
+        <is>
+          <t>BAJWA, RANOLI, LC-246, VASAD, ADAS ROAD, VADOD, LC-258, ANAND Jn, LC-264, KANJARI BORIYAVI, UTARSANDA, NADIAD, LC-278, GOTHAJ, LC-286, MAHEMDABAD AND KHEDA ROAD, LC-294, KANIJ, BAREJADI NANDEJ, GERATPUR, VATVA, KANKARIYA CABIN, AHMEDABAD Jn</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="16" t="inlineStr">
@@ -8944,7 +9308,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M97" s="16" t="inlineStr"/>
+      <c r="M97" s="16" t="inlineStr">
+        <is>
+          <t>BAJWA, RANOLI, LC-246, VASAD, ADAS ROAD, VADOD, LC-258, ANAND Jn, LC-264, KANJARI BORIYAVI, UTARSANDA, NADIAD, LC-278, GOTHAJ, LC-286, MAHEMDABAD AND KHEDA ROAD, LC-294, KANIJ, BAREJADI NANDEJ, GERATPUR, VATVA, KANKARIYA CABIN, AHMEDABAD Jn</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="16" t="inlineStr">
@@ -9001,7 +9369,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M98" s="16" t="inlineStr"/>
+      <c r="M98" s="16" t="inlineStr">
+        <is>
+          <t>BAJWA, RANOLI, LC-246, VASAD, ADAS ROAD, VADOD, LC-258, ANAND Jn, LC-264, KANJARI BORIYAVI, UTARSANDA, NADIAD, LC-278, GOTHAJ, LC-286, MAHEMDABAD AND KHEDA ROAD, LC-294, KANIJ, BAREJADI NANDEJ, GERATPUR, VATVA, KANKARIYA CABIN, AHMEDABAD Jn</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="16" t="inlineStr">
@@ -9058,7 +9430,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M99" s="16" t="inlineStr"/>
+      <c r="M99" s="16" t="inlineStr">
+        <is>
+          <t>BAJWA, RANOLI, LC-246, VASAD, ADAS ROAD, VADOD, LC-258, ANAND Jn, LC-264, KANJARI BORIYAVI, UTARSANDA, NADIAD, LC-278, GOTHAJ, LC-286, MAHEMDABAD AND KHEDA ROAD, LC-294, KANIJ, BAREJADI NANDEJ, GERATPUR, VATVA, KANKARIYA CABIN, AHMEDABAD Jn</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="16" t="inlineStr">
@@ -9115,7 +9491,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M100" s="16" t="inlineStr"/>
+      <c r="M100" s="16" t="inlineStr">
+        <is>
+          <t>BAJWA, RANOLI, LC-246, VASAD, ADAS ROAD, VADOD, LC-258, ANAND Jn, LC-264, KANJARI BORIYAVI, UTARSANDA, NADIAD, LC-278, GOTHAJ, LC-286, MAHEMDABAD AND KHEDA ROAD, LC-294, KANIJ, BAREJADI NANDEJ, GERATPUR, VATVA, KANKARIYA CABIN, AHMEDABAD Jn</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="16" t="inlineStr">
@@ -9172,7 +9552,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M101" s="16" t="inlineStr"/>
+      <c r="M101" s="16" t="inlineStr">
+        <is>
+          <t>BAJWA, RANOLI, LC-246, VASAD, ADAS ROAD, VADOD, LC-258, ANAND Jn, LC-264, KANJARI BORIYAVI, UTARSANDA, NADIAD, LC-278, GOTHAJ, LC-286, MAHEMDABAD AND KHEDA ROAD, LC-294, KANIJ, BAREJADI NANDEJ, GERATPUR, VATVA, KANKARIYA CABIN, AHMEDABAD Jn</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="16" t="inlineStr">
@@ -9229,7 +9613,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M102" s="16" t="inlineStr"/>
+      <c r="M102" s="16" t="inlineStr">
+        <is>
+          <t>BAJWA, RANOLI, LC-246, VASAD, ADAS ROAD, VADOD, LC-258, ANAND Jn, LC-264, KANJARI BORIYAVI, UTARSANDA, NADIAD, LC-278, GOTHAJ, LC-286, MAHEMDABAD AND KHEDA ROAD, LC-294, KANIJ, BAREJADI NANDEJ, GERATPUR, VATVA, KANKARIYA CABIN, AHMEDABAD Jn</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="16" t="inlineStr">
@@ -9286,7 +9674,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M103" s="16" t="inlineStr"/>
+      <c r="M103" s="16" t="inlineStr">
+        <is>
+          <t>BAJWA, RANOLI, LC-246, VASAD, ADAS ROAD, VADOD, LC-258, ANAND Jn, LC-264, KANJARI BORIYAVI, UTARSANDA, NADIAD, LC-278, GOTHAJ, LC-286, MAHEMDABAD AND KHEDA ROAD, LC-294, KANIJ, BAREJADI NANDEJ, GERATPUR, VATVA, KANKARIYA CABIN, AHMEDABAD Jn</t>
+        </is>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="16" t="inlineStr">
@@ -9343,7 +9735,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M104" s="16" t="inlineStr"/>
+      <c r="M104" s="16" t="inlineStr">
+        <is>
+          <t>BAJWA, RANOLI, LC-246, VASAD, ADAS ROAD, VADOD, LC-258, ANAND Jn, LC-264, KANJARI BORIYAVI, UTARSANDA, NADIAD, LC-278, GOTHAJ, LC-286, MAHEMDABAD AND KHEDA ROAD, LC-294, KANIJ, BAREJADI NANDEJ, GERATPUR, VATVA, KANKARIYA CABIN, AHMEDABAD Jn</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="16" t="inlineStr">
@@ -9400,7 +9796,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M105" s="16" t="inlineStr"/>
+      <c r="M105" s="16" t="inlineStr">
+        <is>
+          <t>BAJWA, RANOLI, LC-246, VASAD, ADAS ROAD, VADOD, LC-258, ANAND Jn, LC-264, KANJARI BORIYAVI, UTARSANDA, NADIAD, LC-278, GOTHAJ, LC-286, MAHEMDABAD AND KHEDA ROAD, LC-294, KANIJ, BAREJADI NANDEJ, GERATPUR, VATVA, KANKARIYA CABIN, AHMEDABAD Jn</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="16" t="inlineStr">
@@ -9457,7 +9857,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M106" s="16" t="inlineStr"/>
+      <c r="M106" s="16" t="inlineStr">
+        <is>
+          <t>BAJWA, RANOLI, LC-246, VASAD, ADAS ROAD, VADOD, LC-258, ANAND Jn, LC-264, KANJARI BORIYAVI, UTARSANDA, NADIAD, LC-278, GOTHAJ, LC-286, MAHEMDABAD AND KHEDA ROAD, LC-294, KANIJ, BAREJADI NANDEJ, GERATPUR, VATVA, KANKARIYA CABIN, AHMEDABAD Jn</t>
+        </is>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="16" t="inlineStr">
@@ -9514,7 +9918,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M107" s="16" t="inlineStr"/>
+      <c r="M107" s="16" t="inlineStr">
+        <is>
+          <t>BAJWA, RANOLI, LC-246, VASAD, ADAS ROAD, VADOD, LC-258, ANAND Jn, LC-264, KANJARI BORIYAVI, UTARSANDA, NADIAD, LC-278, GOTHAJ, LC-286, MAHEMDABAD AND KHEDA ROAD, LC-294, KANIJ, BAREJADI NANDEJ, GERATPUR, VATVA, KANKARIYA CABIN, AHMEDABAD Jn</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="16" t="inlineStr">
@@ -9571,7 +9979,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M108" s="16" t="inlineStr"/>
+      <c r="M108" s="16" t="inlineStr">
+        <is>
+          <t>BAJWA, RANOLI, LC-246, VASAD, ADAS ROAD, VADOD, LC-258, ANAND Jn, LC-264, KANJARI BORIYAVI, UTARSANDA, NADIAD, LC-278, GOTHAJ, LC-286, MAHEMDABAD AND KHEDA ROAD, LC-294, KANIJ, BAREJADI NANDEJ, GERATPUR, VATVA, KANKARIYA CABIN, AHMEDABAD Jn</t>
+        </is>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="16" t="inlineStr">
@@ -9628,7 +10040,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M109" s="16" t="inlineStr"/>
+      <c r="M109" s="16" t="inlineStr">
+        <is>
+          <t>BAJWA, RANOLI, LC-246, VASAD, ADAS ROAD, VADOD, LC-258, ANAND Jn, LC-264, KANJARI BORIYAVI, UTARSANDA, NADIAD, LC-278, GOTHAJ, LC-286, MAHEMDABAD AND KHEDA ROAD, LC-294, KANIJ, BAREJADI NANDEJ, GERATPUR, VATVA, KANKARIYA CABIN, AHMEDABAD Jn</t>
+        </is>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="16" t="inlineStr">
@@ -9685,7 +10101,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M110" s="16" t="inlineStr"/>
+      <c r="M110" s="16" t="inlineStr">
+        <is>
+          <t>BAJWA, RANOLI, LC-246, VASAD, ADAS ROAD, VADOD, LC-258, ANAND Jn, LC-264, KANJARI BORIYAVI, UTARSANDA, NADIAD, LC-278, GOTHAJ, LC-286, MAHEMDABAD AND KHEDA ROAD, LC-294, KANIJ, BAREJADI NANDEJ, GERATPUR, VATVA, KANKARIYA CABIN, AHMEDABAD Jn</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="16" t="inlineStr">
@@ -9742,7 +10162,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M111" s="16" t="inlineStr"/>
+      <c r="M111" s="16" t="inlineStr">
+        <is>
+          <t>BAJWA, RANOLI, LC-246, VASAD, ADAS ROAD, VADOD, LC-258, ANAND Jn, LC-264, KANJARI BORIYAVI, UTARSANDA, NADIAD, LC-278, GOTHAJ, LC-286, MAHEMDABAD AND KHEDA ROAD, LC-294, KANIJ, BAREJADI NANDEJ, GERATPUR, VATVA, KANKARIYA CABIN, AHMEDABAD Jn</t>
+        </is>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="31" t="inlineStr">
@@ -9799,7 +10223,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
-      <c r="M112" s="16" t="inlineStr"/>
+      <c r="M112" s="16" t="inlineStr">
+        <is>
+          <t>UTARSANDA, NADIAD, LC-278, GOTHAJ, LC-286, MAHEMDABAD AND KHEDA ROAD, LC-294, KANIJ, BAREJADI NANDEJ, GERATPUR, VATVA, KANKARIYA CABIN, AHMEDABAD Jn</t>
+        </is>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="16" t="inlineStr">
@@ -9856,7 +10284,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M113" s="16" t="inlineStr"/>
+      <c r="M113" s="16" t="inlineStr">
+        <is>
+          <t>BAJWA, RANOLI, LC-246, VASAD, ADAS ROAD, VADOD, LC-258, ANAND Jn, LC-264, KANJARI BORIYAVI, UTARSANDA, NADIAD, LC-278, GOTHAJ, LC-286, MAHEMDABAD AND KHEDA ROAD, LC-294, KANIJ, BAREJADI NANDEJ, GERATPUR, VATVA, KANKARIYA CABIN, AHMEDABAD Jn</t>
+        </is>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="16" t="inlineStr">
@@ -9913,7 +10345,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M114" s="16" t="inlineStr"/>
+      <c r="M114" s="16" t="inlineStr">
+        <is>
+          <t>BAJWA, RANOLI, LC-246, VASAD, ADAS ROAD, VADOD, LC-258, ANAND Jn, LC-264, KANJARI BORIYAVI, UTARSANDA, NADIAD, LC-278, GOTHAJ, LC-286, MAHEMDABAD AND KHEDA ROAD, LC-294, KANIJ, BAREJADI NANDEJ, GERATPUR, VATVA, KANKARIYA CABIN, AHMEDABAD Jn</t>
+        </is>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="31" t="inlineStr">
@@ -9970,7 +10406,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
-      <c r="M115" s="16" t="inlineStr"/>
+      <c r="M115" s="16" t="inlineStr">
+        <is>
+          <t>BAJWA, RANOLI, LC-246, VASAD, ADAS ROAD, VADOD, LC-258, ANAND Jn, LC-264, KANJARI BORIYAVI, UTARSANDA, NADIAD</t>
+        </is>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="31" t="inlineStr">
@@ -10027,7 +10467,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
-      <c r="M116" s="16" t="inlineStr"/>
+      <c r="M116" s="16" t="inlineStr">
+        <is>
+          <t>UTARSANDA, NADIAD, LC-278, GOTHAJ, LC-286, MAHEMDABAD AND KHEDA ROAD, LC-294, KANIJ, BAREJADI NANDEJ, GERATPUR, VATVA, KANKARIYA CABIN, AHMEDABAD Jn</t>
+        </is>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="31" t="inlineStr">
@@ -10084,7 +10528,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
-      <c r="M117" s="16" t="inlineStr"/>
+      <c r="M117" s="16" t="inlineStr">
+        <is>
+          <t>UTARSANDA, NADIAD, LC-278, GOTHAJ, LC-286, MAHEMDABAD AND KHEDA ROAD, LC-294, KANIJ, BAREJADI NANDEJ, GERATPUR, VATVA, KANKARIYA CABIN, AHMEDABAD Jn</t>
+        </is>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="16" t="inlineStr">
@@ -10141,7 +10589,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M118" s="16" t="inlineStr"/>
+      <c r="M118" s="16" t="inlineStr">
+        <is>
+          <t>BAJWA, RANOLI, LC-246, VASAD, ADAS ROAD, VADOD, LC-258, ANAND Jn, LC-264, KANJARI BORIYAVI, UTARSANDA, NADIAD, LC-278, GOTHAJ, LC-286, MAHEMDABAD AND KHEDA ROAD, LC-294, KANIJ, BAREJADI NANDEJ, GERATPUR, VATVA, KANKARIYA CABIN, AHMEDABAD Jn</t>
+        </is>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="31" t="inlineStr">
@@ -10198,7 +10650,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
-      <c r="M119" s="16" t="inlineStr"/>
+      <c r="M119" s="16" t="inlineStr">
+        <is>
+          <t>BAJWA, RANOLI, LC-246, VASAD, ADAS ROAD, VADOD, LC-258, ANAND Jn, LC-264, KANJARI BORIYAVI, UTARSANDA</t>
+        </is>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="16" t="inlineStr">
@@ -10255,7 +10711,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M120" s="16" t="inlineStr"/>
+      <c r="M120" s="16" t="inlineStr">
+        <is>
+          <t>BAJWA, RANOLI, LC-246, VASAD, ADAS ROAD, VADOD, LC-258, ANAND Jn, LC-264, KANJARI BORIYAVI, UTARSANDA, NADIAD, LC-278, GOTHAJ, LC-286, MAHEMDABAD AND KHEDA ROAD, LC-294, KANIJ, BAREJADI NANDEJ, GERATPUR, VATVA, KANKARIYA CABIN, AHMEDABAD Jn</t>
+        </is>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="16" t="inlineStr">
@@ -10312,7 +10772,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M121" s="16" t="inlineStr"/>
+      <c r="M121" s="16" t="inlineStr">
+        <is>
+          <t>BAJWA, RANOLI, LC-246, VASAD, ADAS ROAD, VADOD, LC-258, ANAND Jn, LC-264, KANJARI BORIYAVI, UTARSANDA, NADIAD, LC-278, GOTHAJ, LC-286, MAHEMDABAD AND KHEDA ROAD, LC-294, KANIJ, BAREJADI NANDEJ, GERATPUR, VATVA, KANKARIYA CABIN, AHMEDABAD Jn</t>
+        </is>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="16" t="inlineStr">
@@ -10369,7 +10833,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M122" s="16" t="inlineStr"/>
+      <c r="M122" s="16" t="inlineStr">
+        <is>
+          <t>BAJWA, RANOLI, LC-246, VASAD, ADAS ROAD, VADOD, LC-258, ANAND Jn, LC-264, KANJARI BORIYAVI, UTARSANDA, NADIAD, LC-278, GOTHAJ, LC-286, MAHEMDABAD AND KHEDA ROAD, LC-294, KANIJ, BAREJADI NANDEJ, GERATPUR, VATVA, KANKARIYA CABIN, AHMEDABAD Jn</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>